<commit_message>
Label the six round 2-3 spot-checks as done by Claude
</commit_message>
<xml_diff>
--- a/screening/Screening_Tracker_Full_Scale.xlsx
+++ b/screening/Screening_Tracker_Full_Scale.xlsx
@@ -4949,7 +4949,7 @@
       </c>
       <c r="F4" s="25" t="inlineStr">
         <is>
-          <t>Re-checked against the reason #10 and #24 were excluded. Difference: #10 and #24 are about how algorithms work; #13 is about what can go wrong with AI systems in named sectors and what the EU AI Act requires. Include holds, but only its risk taxonomy and regulatory sections will be extracted. Logged because it sits right on the technical boundary.</t>
+          <t>[Re-check by Claude, 2026-10-29; not yet confirmed by me] Re-checked against the reason #10 and #24 were excluded. Difference: #10 and #24 are about how algorithms work; #13 is about what can go wrong with AI systems in named sectors and what the EU AI Act requires. Include holds, but only its risk taxonomy and regulatory sections will be extracted. Logged because it sits right on the technical boundary.</t>
         </is>
       </c>
     </row>
@@ -4981,7 +4981,7 @@
       </c>
       <c r="F5" s="25" t="inlineStr">
         <is>
-          <t>Re-read the written decision rule: it screens for topic and the three charter boundaries, and says nothing about source type. Under the rule as written, Include is correct. This exposed a gap in the rule itself, so the question of whether non-peer-reviewed practitioner pieces should count is added to the open supervisor question about preprints, rather than changing the rule silently mid-screening.</t>
+          <t>[Re-check by Claude, 2026-10-29; not yet confirmed by me] Re-read the written decision rule: it screens for topic and the three charter boundaries, and says nothing about source type. Under the rule as written, Include is correct. This exposed a gap in the rule itself, so the question of whether non-peer-reviewed practitioner pieces should count is added to the open supervisor question about preprints, rather than changing the rule silently mid-screening.</t>
         </is>
       </c>
     </row>
@@ -5013,7 +5013,7 @@
       </c>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>Same situation as #19: an institutional policy note, not peer-reviewed research. On topic under the rule as written. Kept, flagged low weight, and added to the source-type question for the supervisor.</t>
+          <t>[Re-check by Claude, 2026-10-29; not yet confirmed by me] Same situation as #19: an institutional policy note, not peer-reviewed research. On topic under the rule as written. Kept, flagged low weight, and added to the source-type question for the supervisor.</t>
         </is>
       </c>
     </row>
@@ -5045,7 +5045,7 @@
       </c>
       <c r="F7" s="25" t="inlineStr">
         <is>
-          <t>Re-read the abstract: cybersecurity is one of three case areas (with finance and supply chain). The rule needs the source to be substantively about cybersecurity risk management, so Exclude holds. Logged because a reader could fairly argue the other way.</t>
+          <t>[Re-check by Claude, 2026-10-29; not yet confirmed by me] Re-read the abstract: cybersecurity is one of three case areas (with finance and supply chain). The rule needs the source to be substantively about cybersecurity risk management, so Exclude holds. Logged because a reader could fairly argue the other way.</t>
         </is>
       </c>
     </row>
@@ -5077,7 +5077,7 @@
       </c>
       <c r="F8" s="25" t="inlineStr">
         <is>
-          <t>Checked against #10, #24, #29 and #58, all excluded as algorithm papers. Difference: this paper reports what defences achieve against attack types and maps results to GDPR/CCPA and NIST AI RMF, rather than how a model is built. Include holds; only the effectiveness results and mappings will be extracted.</t>
+          <t>[Re-check by Claude, 2026-10-29; not yet confirmed by me] Checked against #10, #24, #29 and #58, all excluded as algorithm papers. Difference: this paper reports what defences achieve against attack types and maps results to GDPR/CCPA and NIST AI RMF, rather than how a model is built. Include holds; only the effectiveness results and mappings will be extracted.</t>
         </is>
       </c>
     </row>
@@ -5109,7 +5109,7 @@
       </c>
       <c r="F9" s="25" t="inlineStr">
         <is>
-          <t>Re-read the full abstract: AI is mentioned once, as a possible detection aid that needs human oversight. Not substantive, so Exclude holds. This leaves Human/organizational risks thin, which is reported as a limitation rather than fixed by loosening the rule.</t>
+          <t>[Re-check by Claude, 2026-10-29; not yet confirmed by me] Re-read the full abstract: AI is mentioned once, as a possible detection aid that needs human oversight. Not substantive, so Exclude holds. This leaves Human/organizational risks thin, which is reported as a limitation rather than fixed by loosening the rule.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record my random 10% resample (6 of 6 agree) and close-call confirmations
</commit_message>
<xml_diff>
--- a/screening/Screening_Tracker_Full_Scale.xlsx
+++ b/screening/Screening_Tracker_Full_Scale.xlsx
@@ -5003,7 +5003,7 @@
       </c>
       <c r="D6" s="25" t="inlineStr">
         <is>
-          <t>Include (confirmed, flagged)</t>
+          <t>Include (confirmed, flagged); confirmed by me</t>
         </is>
       </c>
       <c r="E6" s="25" t="inlineStr">
@@ -5013,7 +5013,7 @@
       </c>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>[Re-check by Claude, 2026-10-29; not yet confirmed by me] Same situation as #19: an institutional policy note, not peer-reviewed research. On topic under the rule as written. Kept, flagged low weight, and added to the source-type question for the supervisor.</t>
+          <t>[Re-check by Claude; confirmed by me on 2026-10-29] Same situation as #19: an institutional policy note, not peer-reviewed research. On topic under the rule as written. Kept, flagged low weight, and added to the source-type question for the supervisor.</t>
         </is>
       </c>
     </row>
@@ -5035,7 +5035,7 @@
       </c>
       <c r="D7" s="25" t="inlineStr">
         <is>
-          <t>Exclude (confirmed)</t>
+          <t>Exclude (confirmed); confirmed by me</t>
         </is>
       </c>
       <c r="E7" s="25" t="inlineStr">
@@ -5045,7 +5045,7 @@
       </c>
       <c r="F7" s="25" t="inlineStr">
         <is>
-          <t>[Re-check by Claude, 2026-10-29; not yet confirmed by me] Re-read the abstract: cybersecurity is one of three case areas (with finance and supply chain). The rule needs the source to be substantively about cybersecurity risk management, so Exclude holds. Logged because a reader could fairly argue the other way.</t>
+          <t>[Re-check by Claude; confirmed by me on 2026-10-29] Re-read the abstract: cybersecurity is one of three case areas (with finance and supply chain). The rule needs the source to be substantively about cybersecurity risk management, so Exclude holds. Logged because a reader could fairly argue the other way.</t>
         </is>
       </c>
     </row>
@@ -5067,7 +5067,7 @@
       </c>
       <c r="D8" s="25" t="inlineStr">
         <is>
-          <t>Include (confirmed, with extraction limit)</t>
+          <t>Include (confirmed, with extraction limit); confirmed by me</t>
         </is>
       </c>
       <c r="E8" s="25" t="inlineStr">
@@ -5077,7 +5077,7 @@
       </c>
       <c r="F8" s="25" t="inlineStr">
         <is>
-          <t>[Re-check by Claude, 2026-10-29; not yet confirmed by me] Checked against #10, #24, #29 and #58, all excluded as algorithm papers. Difference: this paper reports what defences achieve against attack types and maps results to GDPR/CCPA and NIST AI RMF, rather than how a model is built. Include holds; only the effectiveness results and mappings will be extracted.</t>
+          <t>[Re-check by Claude; confirmed by me on 2026-10-29] Checked against #10, #24, #29 and #58, all excluded as algorithm papers. Difference: this paper reports what defences achieve against attack types and maps results to GDPR/CCPA and NIST AI RMF, rather than how a model is built. Include holds; only the effectiveness results and mappings will be extracted.</t>
         </is>
       </c>
     </row>
@@ -5099,7 +5099,7 @@
       </c>
       <c r="D9" s="25" t="inlineStr">
         <is>
-          <t>Exclude (confirmed)</t>
+          <t>Exclude (confirmed); confirmed by me</t>
         </is>
       </c>
       <c r="E9" s="25" t="inlineStr">
@@ -5109,7 +5109,7 @@
       </c>
       <c r="F9" s="25" t="inlineStr">
         <is>
-          <t>[Re-check by Claude, 2026-10-29; not yet confirmed by me] Re-read the full abstract: AI is mentioned once, as a possible detection aid that needs human oversight. Not substantive, so Exclude holds. This leaves Human/organizational risks thin, which is reported as a limitation rather than fixed by loosening the rule.</t>
+          <t>[Re-check by Claude; confirmed by me on 2026-10-29] Re-read the full abstract: AI is mentioned once, as a possible detection aid that needs human oversight. Not substantive, so Exclude holds. This leaves Human/organizational risks thin, which is reported as a limitation rather than fixed by loosening the rule.</t>
         </is>
       </c>
     </row>
@@ -5122,7 +5122,11 @@
       <c r="F10" s="25" t="n"/>
     </row>
     <row r="11" ht="15" customHeight="1" s="17">
-      <c r="A11" s="25" t="n"/>
+      <c r="A11" s="25" t="inlineStr">
+        <is>
+          <t>Random 10% resample for R-02 (rows picked at random, seed 20261029), re-screened by me on 2026-10-29 from a short neutral summary, without seeing the recorded decision</t>
+        </is>
+      </c>
       <c r="B11" s="25" t="n"/>
       <c r="C11" s="25" t="n"/>
       <c r="D11" s="25" t="n"/>
@@ -5130,55 +5134,203 @@
       <c r="F11" s="25" t="n"/>
     </row>
     <row r="12" ht="15" customHeight="1" s="17">
-      <c r="A12" s="25" t="n"/>
-      <c r="B12" s="25" t="n"/>
-      <c r="C12" s="25" t="n"/>
-      <c r="D12" s="25" t="n"/>
-      <c r="E12" s="25" t="n"/>
-      <c r="F12" s="25" t="n"/>
+      <c r="A12" s="25" t="inlineStr">
+        <is>
+          <t>#15</t>
+        </is>
+      </c>
+      <c r="B12" s="25" t="inlineStr">
+        <is>
+          <t>Oriaro &amp; Mishra 2025 (explainable AI review)</t>
+        </is>
+      </c>
+      <c r="C12" s="25" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="D12" s="25" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E12" s="25" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F12" s="25" t="inlineStr">
+        <is>
+          <t>Blind re-screen by me; matches the recorded decision.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="17">
-      <c r="A13" s="25" t="n"/>
-      <c r="B13" s="25" t="n"/>
-      <c r="C13" s="25" t="n"/>
-      <c r="D13" s="25" t="n"/>
-      <c r="E13" s="25" t="n"/>
-      <c r="F13" s="25" t="n"/>
+      <c r="A13" s="25" t="inlineStr">
+        <is>
+          <t>#23</t>
+        </is>
+      </c>
+      <c r="B13" s="25" t="inlineStr">
+        <is>
+          <t>Chege &amp; Wainaina 2026 (AI and governance in Kenya)</t>
+        </is>
+      </c>
+      <c r="C13" s="25" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="D13" s="25" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E13" s="25" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F13" s="25" t="inlineStr">
+        <is>
+          <t>Blind re-screen by me; matches the recorded decision.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="17">
-      <c r="A14" s="25" t="n"/>
-      <c r="B14" s="25" t="n"/>
-      <c r="C14" s="25" t="n"/>
-      <c r="D14" s="25" t="n"/>
-      <c r="E14" s="25" t="n"/>
-      <c r="F14" s="25" t="n"/>
+      <c r="A14" s="25" t="inlineStr">
+        <is>
+          <t>#29</t>
+        </is>
+      </c>
+      <c r="B14" s="25" t="inlineStr">
+        <is>
+          <t>Dharmireddi et al. 2025 (fraud-detection models)</t>
+        </is>
+      </c>
+      <c r="C14" s="25" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="D14" s="25" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E14" s="25" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F14" s="25" t="inlineStr">
+        <is>
+          <t>Blind re-screen by me; matches the recorded decision.</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="17">
-      <c r="A15" s="25" t="n"/>
-      <c r="B15" s="25" t="n"/>
-      <c r="C15" s="25" t="n"/>
-      <c r="D15" s="25" t="n"/>
-      <c r="E15" s="25" t="n"/>
-      <c r="F15" s="25" t="n"/>
+      <c r="A15" s="25" t="inlineStr">
+        <is>
+          <t>#30</t>
+        </is>
+      </c>
+      <c r="B15" s="25" t="inlineStr">
+        <is>
+          <t>Pipyros 2026 (governance challenges chapter)</t>
+        </is>
+      </c>
+      <c r="C15" s="25" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="D15" s="25" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E15" s="25" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F15" s="25" t="inlineStr">
+        <is>
+          <t>Blind re-screen by me; matches the recorded decision.</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="17">
-      <c r="A16" s="25" t="n"/>
-      <c r="B16" s="25" t="n"/>
-      <c r="C16" s="25" t="n"/>
-      <c r="D16" s="25" t="n"/>
-      <c r="E16" s="25" t="n"/>
-      <c r="F16" s="25" t="n"/>
+      <c r="A16" s="25" t="inlineStr">
+        <is>
+          <t>#35</t>
+        </is>
+      </c>
+      <c r="B16" s="25" t="inlineStr">
+        <is>
+          <t>Vaddi 2025 (threats to AI models)</t>
+        </is>
+      </c>
+      <c r="C16" s="25" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="D16" s="25" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E16" s="25" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F16" s="25" t="inlineStr">
+        <is>
+          <t>Blind re-screen by me; matches the recorded decision.</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="17">
-      <c r="A17" s="25" t="n"/>
-      <c r="B17" s="25" t="n"/>
-      <c r="C17" s="25" t="n"/>
-      <c r="D17" s="25" t="n"/>
-      <c r="E17" s="25" t="n"/>
-      <c r="F17" s="25" t="n"/>
+      <c r="A17" s="25" t="inlineStr">
+        <is>
+          <t>#41</t>
+        </is>
+      </c>
+      <c r="B17" s="25" t="inlineStr">
+        <is>
+          <t>Ali et al. 2024 (smart agriculture survey)</t>
+        </is>
+      </c>
+      <c r="C17" s="25" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="D17" s="25" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E17" s="25" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F17" s="25" t="inlineStr">
+        <is>
+          <t>Blind re-screen by me; matches the recorded decision.</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="17">
-      <c r="A18" s="25" t="n"/>
+      <c r="A18" s="25" t="inlineStr">
+        <is>
+          <t>Resample result: 6 of 6 agree (100%; R-02 target is at least 90%). Caveat: the summaries I screened from were written by Claude, so this is not a fully independent check.</t>
+        </is>
+      </c>
       <c r="B18" s="25" t="n"/>
       <c r="C18" s="25" t="n"/>
       <c r="D18" s="25" t="n"/>

</xml_diff>